<commit_message>
Import products only (into a store); add pull-to-refresh on all screens
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01D4ykufBtDCW4pyrDqaW8UA
</commit_message>
<xml_diff>
--- a/templates/import_template.xlsx
+++ b/templates/import_template.xlsx
@@ -59,9 +59,7 @@
   </cellStyleXfs>
   <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -428,56 +426,38 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H6"/>
+  <dimension ref="A1:E5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="18" customWidth="1" min="1" max="1"/>
-    <col width="20" customWidth="1" min="2" max="2"/>
-    <col width="32" customWidth="1" min="3" max="3"/>
-    <col width="22" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="10" customWidth="1" min="6" max="6"/>
-    <col width="10" customWidth="1" min="7" max="7"/>
-    <col width="24" customWidth="1" min="8" max="8"/>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="28" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Company</t>
+          <t>Product</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Store</t>
+          <t>SKU</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Store Address</t>
+          <t>Price</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Product</t>
+          <t>Quantity</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>SKU</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>Price</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>Quantity</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Description</t>
         </is>
@@ -486,36 +466,21 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Acme Ltd</t>
+          <t>Blue Widget</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Hull City Centre</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>12 Whitefriargate, Hull HU1 2HA</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>Blue Widget</t>
-        </is>
+          <t>AC-001</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="n">
+        <v>4.99</v>
+      </c>
+      <c r="D2" t="n">
+        <v>120</v>
       </c>
       <c r="E2" t="inlineStr">
-        <is>
-          <t>AC-001</t>
-        </is>
-      </c>
-      <c r="F2" s="2" t="n">
-        <v>4.99</v>
-      </c>
-      <c r="G2" t="n">
-        <v>120</v>
-      </c>
-      <c r="H2" t="inlineStr">
         <is>
           <t>Standard size</t>
         </is>
@@ -524,134 +489,63 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Acme Ltd</t>
+          <t>Red Widget</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Hull City Centre</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr"/>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>Red Widget</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
           <t>AC-002</t>
         </is>
       </c>
-      <c r="F3" s="2" t="n">
+      <c r="C3" s="2" t="n">
         <v>5.49</v>
       </c>
-      <c r="G3" t="n">
+      <c r="D3" t="n">
         <v>80</v>
       </c>
-      <c r="H3" t="inlineStr"/>
+      <c r="E3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Acme Ltd</t>
+          <t>Oat Milk 1L</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Leeds Trinity</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>Trinity Leeds, LS1 5AT</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>Blue Widget</t>
-        </is>
+          <t>NF-OM1</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="n">
+        <v>1.85</v>
+      </c>
+      <c r="D4" t="n">
+        <v>200</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>AC-001</t>
-        </is>
-      </c>
-      <c r="F4" s="2" t="n">
-        <v>4.99</v>
-      </c>
-      <c r="G4" t="n">
-        <v>45</v>
-      </c>
-      <c r="H4" t="inlineStr"/>
+          <t>Barista edition</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Northern Foods</t>
+          <t>Granola 500g</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>York Shambles</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>5 The Shambles, York YO1 7LX</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>Oat Milk 1L</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>NF-OM1</t>
-        </is>
-      </c>
-      <c r="F5" s="2" t="n">
-        <v>1.85</v>
-      </c>
-      <c r="G5" t="n">
-        <v>200</v>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>Barista edition</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Northern Foods</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>York Shambles</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr"/>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>Granola 500g</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
           <t>NF-GR5</t>
         </is>
       </c>
-      <c r="F6" s="2" t="n">
+      <c r="C5" s="2" t="n">
         <v>3.2</v>
       </c>
-      <c r="G6" t="n">
+      <c r="D5" t="n">
         <v>60</v>
       </c>
-      <c r="H6" t="inlineStr"/>
+      <c r="E5" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Three prices per product: retail (staff read-only), wholesale and per item (admin only)
- Retail stored on the product (retailPrice): everyone signed in can read, only admins change
- Wholesale/per item stored in admin-only productPrices collection
- Old single price migrates to retail automatically on admin sign-in
- Product form, store cards, tables/PDF, barcode fill, Excel import updated
- Firestore rules: productPrices admin-only; retailPrice validated

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01D4ykufBtDCW4pyrDqaW8UA
</commit_message>
<xml_diff>
--- a/templates/import_template.xlsx
+++ b/templates/import_template.xlsx
@@ -57,9 +57,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -426,14 +427,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E5"/>
+  <dimension ref="A1:G5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="24" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="10" customWidth="1" min="4" max="4"/>
-    <col width="28" customWidth="1" min="5" max="5"/>
+    <col width="36" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="26" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -449,15 +452,25 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Price</t>
+          <t>Retail Price</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
+          <t>Wholesale Price</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Per Item Price</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
           <t>Quantity</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Description</t>
         </is>
@@ -466,86 +479,106 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Blue Widget</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>AC-001</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="n">
-        <v>4.99</v>
-      </c>
-      <c r="D2" t="n">
-        <v>120</v>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>Standard size</t>
-        </is>
-      </c>
+          <t>Garnier Micellar Water 400ml</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>3600542024453</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="n">
+        <v>6.99</v>
+      </c>
+      <c r="D2" s="3" t="n">
+        <v>4.2</v>
+      </c>
+      <c r="E2" s="3" t="n">
+        <v>7.49</v>
+      </c>
+      <c r="F2" t="n">
+        <v>48</v>
+      </c>
+      <c r="G2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Red Widget</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>AC-002</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="n">
-        <v>5.49</v>
-      </c>
-      <c r="D3" t="n">
-        <v>80</v>
-      </c>
-      <c r="E3" t="inlineStr"/>
+          <t>Nivea Soft Cream 200ml</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>4005808890507</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="D3" s="3" t="n">
+        <v>2.75</v>
+      </c>
+      <c r="E3" s="3" t="n">
+        <v>4.99</v>
+      </c>
+      <c r="F3" t="n">
+        <v>36</v>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Moisturising cream</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Oat Milk 1L</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>NF-OM1</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="n">
-        <v>1.85</v>
-      </c>
-      <c r="D4" t="n">
-        <v>200</v>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>Barista edition</t>
-        </is>
-      </c>
+          <t>Maybelline Lash Sensational Mascara</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>3600531139582</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="n">
+        <v>11.99</v>
+      </c>
+      <c r="D4" s="3" t="n">
+        <v>7.1</v>
+      </c>
+      <c r="E4" s="3" t="n">
+        <v>12.99</v>
+      </c>
+      <c r="F4" t="n">
+        <v>24</v>
+      </c>
+      <c r="G4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Granola 500g</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>NF-GR5</t>
-        </is>
-      </c>
-      <c r="C5" s="2" t="n">
-        <v>3.2</v>
-      </c>
-      <c r="D5" t="n">
+          <t>Dove Original Deodorant 250ml</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>8710447313383</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="n">
+        <v>3.25</v>
+      </c>
+      <c r="D5" s="3" t="n">
+        <v>1.95</v>
+      </c>
+      <c r="E5" s="3" t="n">
+        <v>3.49</v>
+      </c>
+      <c r="F5" t="n">
         <v>60</v>
       </c>
-      <c r="E5" t="inlineStr"/>
+      <c r="G5" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Prevent duplicate SKUs per store; low-stock reorder warnings
- 'Product already exists' prompt on scan and on save; duplicates blocked per store
- Store scan shows 'already exists' and opens the product
- Reorder level per product (default 5): amber 'Needs ordering', red 'Out of stock'
- Needs-ordering banners on home, company and store pages with filters
- Tables: Stock status column, highlighted rows, 'Needs ordering only' filter
- Excel import: Reorder Level column; rules validate reorderLevel

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01D4ykufBtDCW4pyrDqaW8UA
</commit_message>
<xml_diff>
--- a/templates/import_template.xlsx
+++ b/templates/import_template.xlsx
@@ -41,7 +41,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="002357D9"/>
+        <fgColor rgb="005B1F52"/>
       </patternFill>
     </fill>
   </fills>
@@ -57,10 +57,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -427,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G5"/>
+  <dimension ref="A1:H5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="36" customWidth="1" min="1" max="1"/>
@@ -436,7 +435,8 @@
     <col width="16" customWidth="1" min="4" max="4"/>
     <col width="15" customWidth="1" min="5" max="5"/>
     <col width="10" customWidth="1" min="6" max="6"/>
-    <col width="26" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="26" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -472,6 +472,11 @@
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
+          <t>Reorder Level</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
           <t>Description</t>
         </is>
       </c>
@@ -482,24 +487,27 @@
           <t>Garnier Micellar Water 400ml</t>
         </is>
       </c>
-      <c r="B2" s="2" t="inlineStr">
+      <c r="B2" t="inlineStr">
         <is>
           <t>3600542024453</t>
         </is>
       </c>
-      <c r="C2" s="3" t="n">
+      <c r="C2" s="2" t="n">
         <v>6.99</v>
       </c>
-      <c r="D2" s="3" t="n">
+      <c r="D2" s="2" t="n">
         <v>4.2</v>
       </c>
-      <c r="E2" s="3" t="n">
+      <c r="E2" s="2" t="n">
         <v>7.49</v>
       </c>
       <c r="F2" t="n">
         <v>48</v>
       </c>
-      <c r="G2" t="inlineStr"/>
+      <c r="G2" t="n">
+        <v>10</v>
+      </c>
+      <c r="H2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -507,24 +515,27 @@
           <t>Nivea Soft Cream 200ml</t>
         </is>
       </c>
-      <c r="B3" s="2" t="inlineStr">
+      <c r="B3" t="inlineStr">
         <is>
           <t>4005808890507</t>
         </is>
       </c>
-      <c r="C3" s="3" t="n">
+      <c r="C3" s="2" t="n">
         <v>4.5</v>
       </c>
-      <c r="D3" s="3" t="n">
+      <c r="D3" s="2" t="n">
         <v>2.75</v>
       </c>
-      <c r="E3" s="3" t="n">
+      <c r="E3" s="2" t="n">
         <v>4.99</v>
       </c>
       <c r="F3" t="n">
         <v>36</v>
       </c>
-      <c r="G3" t="inlineStr">
+      <c r="G3" t="n">
+        <v>8</v>
+      </c>
+      <c r="H3" t="inlineStr">
         <is>
           <t>Moisturising cream</t>
         </is>
@@ -536,24 +547,27 @@
           <t>Maybelline Lash Sensational Mascara</t>
         </is>
       </c>
-      <c r="B4" s="2" t="inlineStr">
+      <c r="B4" t="inlineStr">
         <is>
           <t>3600531139582</t>
         </is>
       </c>
-      <c r="C4" s="3" t="n">
+      <c r="C4" s="2" t="n">
         <v>11.99</v>
       </c>
-      <c r="D4" s="3" t="n">
+      <c r="D4" s="2" t="n">
         <v>7.1</v>
       </c>
-      <c r="E4" s="3" t="n">
+      <c r="E4" s="2" t="n">
         <v>12.99</v>
       </c>
       <c r="F4" t="n">
-        <v>24</v>
-      </c>
-      <c r="G4" t="inlineStr"/>
+        <v>4</v>
+      </c>
+      <c r="G4" t="n">
+        <v>6</v>
+      </c>
+      <c r="H4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -561,24 +575,24 @@
           <t>Dove Original Deodorant 250ml</t>
         </is>
       </c>
-      <c r="B5" s="2" t="inlineStr">
+      <c r="B5" t="inlineStr">
         <is>
           <t>8710447313383</t>
         </is>
       </c>
-      <c r="C5" s="3" t="n">
+      <c r="C5" s="2" t="n">
         <v>3.25</v>
       </c>
-      <c r="D5" s="3" t="n">
+      <c r="D5" s="2" t="n">
         <v>1.95</v>
       </c>
-      <c r="E5" s="3" t="n">
+      <c r="E5" s="2" t="n">
         <v>3.49</v>
       </c>
       <c r="F5" t="n">
         <v>60</v>
       </c>
-      <c r="G5" t="inlineStr"/>
+      <c r="H5" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Currency: Qatari riyal (QAR) instead of GBP
- money() formats as 'QAR 1,234.50' across app, tables and PDFs
- Price fields show QAR prefix; shared parseMoney accepts QAR / ر.ق / ريال / plain numbers
- Import templates use QAR prices and number format

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01D4ykufBtDCW4pyrDqaW8UA
</commit_message>
<xml_diff>
--- a/templates/import_template.xlsx
+++ b/templates/import_template.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="£#,##0.00"/>
+    <numFmt numFmtId="164" formatCode="&quot;QAR &quot;#,##0.00"/>
   </numFmts>
   <fonts count="2">
     <font>
@@ -431,9 +431,9 @@
   <cols>
     <col width="36" customWidth="1" min="1" max="1"/>
     <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="15" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="17" customWidth="1" min="5" max="5"/>
     <col width="10" customWidth="1" min="6" max="6"/>
     <col width="14" customWidth="1" min="7" max="7"/>
     <col width="26" customWidth="1" min="8" max="8"/>
@@ -493,13 +493,13 @@
         </is>
       </c>
       <c r="C2" s="2" t="n">
-        <v>6.99</v>
+        <v>32</v>
       </c>
       <c r="D2" s="2" t="n">
-        <v>4.2</v>
+        <v>19.5</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>7.49</v>
+        <v>34.5</v>
       </c>
       <c r="F2" t="n">
         <v>48</v>
@@ -521,13 +521,13 @@
         </is>
       </c>
       <c r="C3" s="2" t="n">
-        <v>4.5</v>
+        <v>21</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>2.75</v>
+        <v>12.75</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>4.99</v>
+        <v>23</v>
       </c>
       <c r="F3" t="n">
         <v>36</v>
@@ -553,13 +553,13 @@
         </is>
       </c>
       <c r="C4" s="2" t="n">
-        <v>11.99</v>
+        <v>55</v>
       </c>
       <c r="D4" s="2" t="n">
-        <v>7.1</v>
+        <v>32.5</v>
       </c>
       <c r="E4" s="2" t="n">
-        <v>12.99</v>
+        <v>59</v>
       </c>
       <c r="F4" t="n">
         <v>4</v>
@@ -581,13 +581,13 @@
         </is>
       </c>
       <c r="C5" s="2" t="n">
-        <v>3.25</v>
+        <v>15</v>
       </c>
       <c r="D5" s="2" t="n">
-        <v>1.95</v>
+        <v>9</v>
       </c>
       <c r="E5" s="2" t="n">
-        <v>3.49</v>
+        <v>16</v>
       </c>
       <c r="F5" t="n">
         <v>60</v>

</xml_diff>

<commit_message>
Prices are now Cost, Wholesale and Retail (QAR)
- 'Per item' price replaced by Cost price (admin-only, stored in productPrices)
- Retail stays visible (read-only) to staff; cost and wholesale admin-only
- Product form, cards, tables/PDF, Excel import and templates updated

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01D4ykufBtDCW4pyrDqaW8UA
</commit_message>
<xml_diff>
--- a/templates/import_template.xlsx
+++ b/templates/import_template.xlsx
@@ -431,9 +431,9 @@
   <cols>
     <col width="36" customWidth="1" min="1" max="1"/>
     <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
-    <col width="17" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="17" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
     <col width="10" customWidth="1" min="6" max="6"/>
     <col width="14" customWidth="1" min="7" max="7"/>
     <col width="26" customWidth="1" min="8" max="8"/>
@@ -452,17 +452,17 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
+          <t>Cost Price</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Wholesale Price</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
           <t>Retail Price</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>Wholesale Price</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>Per Item Price</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
@@ -493,13 +493,13 @@
         </is>
       </c>
       <c r="C2" s="2" t="n">
-        <v>32</v>
+        <v>14</v>
       </c>
       <c r="D2" s="2" t="n">
         <v>19.5</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>34.5</v>
+        <v>32</v>
       </c>
       <c r="F2" t="n">
         <v>48</v>
@@ -521,13 +521,13 @@
         </is>
       </c>
       <c r="C3" s="2" t="n">
-        <v>21</v>
+        <v>9.5</v>
       </c>
       <c r="D3" s="2" t="n">
         <v>12.75</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="F3" t="n">
         <v>36</v>
@@ -553,13 +553,13 @@
         </is>
       </c>
       <c r="C4" s="2" t="n">
-        <v>55</v>
+        <v>24</v>
       </c>
       <c r="D4" s="2" t="n">
         <v>32.5</v>
       </c>
       <c r="E4" s="2" t="n">
-        <v>59</v>
+        <v>55</v>
       </c>
       <c r="F4" t="n">
         <v>4</v>
@@ -581,13 +581,13 @@
         </is>
       </c>
       <c r="C5" s="2" t="n">
-        <v>15</v>
+        <v>6.5</v>
       </c>
       <c r="D5" s="2" t="n">
         <v>9</v>
       </c>
       <c r="E5" s="2" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="F5" t="n">
         <v>60</v>

</xml_diff>